<commit_message>
Estimar los días libres como un día típico de 3 Ubers
Los días libres usaban el promedio de un día de agenda, que tiene más
traslados y más largos. Ahora se estiman como 2 lugares y vuelta
(3 Ubers de unos 10 km), con la cantidad de Ubers ajustable.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/viajes-uber-la.xlsx
+++ b/viajes-uber-la.xlsx
@@ -538,13 +538,12 @@
           <t>Gasto por día libre</t>
         </is>
       </c>
-      <c r="C6" s="5">
-        <f>ROUND(AVERAGE(E12,E13,E14,E16),0)</f>
-        <v/>
+      <c r="C6" s="5" t="n">
+        <v>149</v>
       </c>
       <c r="E6" s="3" t="inlineStr">
         <is>
-          <t>Por defecto: promedio de un día en LA (días 1, 2, 3 y 5). Escribí otro monto para cambiarlo.</t>
+          <t>Día libre típico: 2 lugares = 3 Ubers de unos 10 km (≈ US$ 50 cada uno). Escribí otro monto para cambiarlo.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Tarjetas sobre el mapa en el celular y UberXXL para el aeropuerto
En la vista Mapa del celular hay tarjetas deslizables con cada actividad
y su traslado; al tocarlas o deslizarlas se marca el lugar y el tramo en
el mapa. La llegada y la ida al aeropuerto pasan a UberXXL por las
valijas (15 % sobre XL).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/viajes-uber-la.xlsx
+++ b/viajes-uber-la.xlsx
@@ -586,7 +586,7 @@
         </is>
       </c>
       <c r="D9" s="8">
-        <f>COUNTIFS(Viajes!$A$2:$A$26,B9,Viajes!$E$2:$E$26,"UberXL")</f>
+        <f>COUNTIFS(Viajes!$A$2:$A$26,B9,Viajes!$E$2:$E$26,"Uber*")</f>
         <v/>
       </c>
       <c r="E9" s="9">
@@ -609,7 +609,7 @@
         </is>
       </c>
       <c r="D10" s="11">
-        <f>COUNTIFS(Viajes!$A$2:$A$26,B10,Viajes!$E$2:$E$26,"UberXL")</f>
+        <f>COUNTIFS(Viajes!$A$2:$A$26,B10,Viajes!$E$2:$E$26,"Uber*")</f>
         <v/>
       </c>
       <c r="E10" s="12">
@@ -632,7 +632,7 @@
         </is>
       </c>
       <c r="D11" s="11">
-        <f>COUNTIFS(Viajes!$A$2:$A$26,B11,Viajes!$E$2:$E$26,"UberXL")</f>
+        <f>COUNTIFS(Viajes!$A$2:$A$26,B11,Viajes!$E$2:$E$26,"Uber*")</f>
         <v/>
       </c>
       <c r="E11" s="12">
@@ -655,7 +655,7 @@
         </is>
       </c>
       <c r="D12" s="8">
-        <f>COUNTIFS(Viajes!$A$2:$A$26,B12,Viajes!$E$2:$E$26,"UberXL")</f>
+        <f>COUNTIFS(Viajes!$A$2:$A$26,B12,Viajes!$E$2:$E$26,"Uber*")</f>
         <v/>
       </c>
       <c r="E12" s="9">
@@ -678,7 +678,7 @@
         </is>
       </c>
       <c r="D13" s="8">
-        <f>COUNTIFS(Viajes!$A$2:$A$26,B13,Viajes!$E$2:$E$26,"UberXL")</f>
+        <f>COUNTIFS(Viajes!$A$2:$A$26,B13,Viajes!$E$2:$E$26,"Uber*")</f>
         <v/>
       </c>
       <c r="E13" s="9">
@@ -701,7 +701,7 @@
         </is>
       </c>
       <c r="D14" s="8">
-        <f>COUNTIFS(Viajes!$A$2:$A$26,B14,Viajes!$E$2:$E$26,"UberXL")</f>
+        <f>COUNTIFS(Viajes!$A$2:$A$26,B14,Viajes!$E$2:$E$26,"Uber*")</f>
         <v/>
       </c>
       <c r="E14" s="9">
@@ -724,7 +724,7 @@
         </is>
       </c>
       <c r="D15" s="8">
-        <f>COUNTIFS(Viajes!$A$2:$A$26,B15,Viajes!$E$2:$E$26,"UberXL")</f>
+        <f>COUNTIFS(Viajes!$A$2:$A$26,B15,Viajes!$E$2:$E$26,"Uber*")</f>
         <v/>
       </c>
       <c r="E15" s="9">
@@ -747,7 +747,7 @@
         </is>
       </c>
       <c r="D16" s="8">
-        <f>COUNTIFS(Viajes!$A$2:$A$26,B16,Viajes!$E$2:$E$26,"UberXL")</f>
+        <f>COUNTIFS(Viajes!$A$2:$A$26,B16,Viajes!$E$2:$E$26,"Uber*")</f>
         <v/>
       </c>
       <c r="E16" s="9">
@@ -770,7 +770,7 @@
         </is>
       </c>
       <c r="D17" s="8">
-        <f>COUNTIFS(Viajes!$A$2:$A$26,B17,Viajes!$E$2:$E$26,"UberXL")</f>
+        <f>COUNTIFS(Viajes!$A$2:$A$26,B17,Viajes!$E$2:$E$26,"Uber*")</f>
         <v/>
       </c>
       <c r="E17" s="9">
@@ -793,7 +793,7 @@
         </is>
       </c>
       <c r="D18" s="11">
-        <f>COUNTIFS(Viajes!$A$2:$A$26,B18,Viajes!$E$2:$E$26,"UberXL")</f>
+        <f>COUNTIFS(Viajes!$A$2:$A$26,B18,Viajes!$E$2:$E$26,"Uber*")</f>
         <v/>
       </c>
       <c r="E18" s="12">
@@ -816,7 +816,7 @@
         </is>
       </c>
       <c r="D19" s="11">
-        <f>COUNTIFS(Viajes!$A$2:$A$26,B19,Viajes!$E$2:$E$26,"UberXL")</f>
+        <f>COUNTIFS(Viajes!$A$2:$A$26,B19,Viajes!$E$2:$E$26,"Uber*")</f>
         <v/>
       </c>
       <c r="E19" s="12">
@@ -839,7 +839,7 @@
         </is>
       </c>
       <c r="D20" s="11">
-        <f>COUNTIFS(Viajes!$A$2:$A$26,B20,Viajes!$E$2:$E$26,"UberXL")</f>
+        <f>COUNTIFS(Viajes!$A$2:$A$26,B20,Viajes!$E$2:$E$26,"Uber*")</f>
         <v/>
       </c>
       <c r="E20" s="12">
@@ -862,7 +862,7 @@
         </is>
       </c>
       <c r="D21" s="11">
-        <f>COUNTIFS(Viajes!$A$2:$A$26,B21,Viajes!$E$2:$E$26,"UberXL")</f>
+        <f>COUNTIFS(Viajes!$A$2:$A$26,B21,Viajes!$E$2:$E$26,"Uber*")</f>
         <v/>
       </c>
       <c r="E21" s="12">
@@ -885,7 +885,7 @@
         </is>
       </c>
       <c r="D22" s="8">
-        <f>COUNTIFS(Viajes!$A$2:$A$26,B22,Viajes!$E$2:$E$26,"UberXL")</f>
+        <f>COUNTIFS(Viajes!$A$2:$A$26,B22,Viajes!$E$2:$E$26,"Uber*")</f>
         <v/>
       </c>
       <c r="E22" s="9">
@@ -1101,7 +1101,7 @@
       </c>
       <c r="E2" s="8" t="inlineStr">
         <is>
-          <t>UberXL</t>
+          <t>UberXXL</t>
         </is>
       </c>
       <c r="F2" s="18" t="n">
@@ -1126,10 +1126,10 @@
         <v>50</v>
       </c>
       <c r="M2" s="9" t="n">
-        <v>87.70999999999999</v>
+        <v>100.87</v>
       </c>
       <c r="N2" s="9">
-        <f>IF(E2="UberXL",M2*(1+Resumen!$C$5),0)</f>
+        <f>IF(LEFT(E2,4)="Uber",M2*(1+Resumen!$C$5),0)</f>
         <v/>
       </c>
       <c r="O2" s="21" t="n"/>
@@ -1194,7 +1194,7 @@
         <v>43.46</v>
       </c>
       <c r="N3" s="9">
-        <f>IF(E3="UberXL",M3*(1+Resumen!$C$5),0)</f>
+        <f>IF(LEFT(E3,4)="Uber",M3*(1+Resumen!$C$5),0)</f>
         <v/>
       </c>
       <c r="O3" s="21" t="n"/>
@@ -1259,7 +1259,7 @@
         <v>71.31999999999999</v>
       </c>
       <c r="N4" s="9">
-        <f>IF(E4="UberXL",M4*(1+Resumen!$C$5),0)</f>
+        <f>IF(LEFT(E4,4)="Uber",M4*(1+Resumen!$C$5),0)</f>
         <v/>
       </c>
       <c r="O4" s="21" t="n"/>
@@ -1322,7 +1322,7 @@
         <v>0</v>
       </c>
       <c r="N5" s="9">
-        <f>IF(E5="UberXL",M5*(1+Resumen!$C$5),0)</f>
+        <f>IF(LEFT(E5,4)="Uber",M5*(1+Resumen!$C$5),0)</f>
         <v/>
       </c>
       <c r="O5" s="21" t="n"/>
@@ -1387,7 +1387,7 @@
         <v>49.19</v>
       </c>
       <c r="N6" s="9">
-        <f>IF(E6="UberXL",M6*(1+Resumen!$C$5),0)</f>
+        <f>IF(LEFT(E6,4)="Uber",M6*(1+Resumen!$C$5),0)</f>
         <v/>
       </c>
       <c r="O6" s="21" t="n"/>
@@ -1450,7 +1450,7 @@
         <v>24</v>
       </c>
       <c r="N7" s="9">
-        <f>IF(E7="UberXL",M7*(1+Resumen!$C$5),0)</f>
+        <f>IF(LEFT(E7,4)="Uber",M7*(1+Resumen!$C$5),0)</f>
         <v/>
       </c>
       <c r="O7" s="21" t="n"/>
@@ -1515,7 +1515,7 @@
         <v>25.45</v>
       </c>
       <c r="N8" s="9">
-        <f>IF(E8="UberXL",M8*(1+Resumen!$C$5),0)</f>
+        <f>IF(LEFT(E8,4)="Uber",M8*(1+Resumen!$C$5),0)</f>
         <v/>
       </c>
       <c r="O8" s="21" t="n"/>
@@ -1580,7 +1580,7 @@
         <v>51.83</v>
       </c>
       <c r="N9" s="9">
-        <f>IF(E9="UberXL",M9*(1+Resumen!$C$5),0)</f>
+        <f>IF(LEFT(E9,4)="Uber",M9*(1+Resumen!$C$5),0)</f>
         <v/>
       </c>
       <c r="O9" s="21" t="n"/>
@@ -1649,7 +1649,7 @@
         <v>57.88</v>
       </c>
       <c r="N10" s="9">
-        <f>IF(E10="UberXL",M10*(1+Resumen!$C$5),0)</f>
+        <f>IF(LEFT(E10,4)="Uber",M10*(1+Resumen!$C$5),0)</f>
         <v/>
       </c>
       <c r="O10" s="21" t="n"/>
@@ -1716,7 +1716,7 @@
         <v>24</v>
       </c>
       <c r="N11" s="9">
-        <f>IF(E11="UberXL",M11*(1+Resumen!$C$5),0)</f>
+        <f>IF(LEFT(E11,4)="Uber",M11*(1+Resumen!$C$5),0)</f>
         <v/>
       </c>
       <c r="O11" s="21" t="n"/>
@@ -1781,7 +1781,7 @@
         <v>38.05</v>
       </c>
       <c r="N12" s="9">
-        <f>IF(E12="UberXL",M12*(1+Resumen!$C$5),0)</f>
+        <f>IF(LEFT(E12,4)="Uber",M12*(1+Resumen!$C$5),0)</f>
         <v/>
       </c>
       <c r="O12" s="21" t="n"/>
@@ -1846,7 +1846,7 @@
         <v>114.84</v>
       </c>
       <c r="N13" s="9">
-        <f>IF(E13="UberXL",M13*(1+Resumen!$C$5),0)</f>
+        <f>IF(LEFT(E13,4)="Uber",M13*(1+Resumen!$C$5),0)</f>
         <v/>
       </c>
       <c r="O13" s="21" t="n"/>
@@ -1909,7 +1909,7 @@
         <v>61.07</v>
       </c>
       <c r="N14" s="9">
-        <f>IF(E14="UberXL",M14*(1+Resumen!$C$5),0)</f>
+        <f>IF(LEFT(E14,4)="Uber",M14*(1+Resumen!$C$5),0)</f>
         <v/>
       </c>
       <c r="O14" s="21" t="n"/>
@@ -1974,7 +1974,7 @@
         <v>129.15</v>
       </c>
       <c r="N15" s="9">
-        <f>IF(E15="UberXL",M15*(1+Resumen!$C$5),0)</f>
+        <f>IF(LEFT(E15,4)="Uber",M15*(1+Resumen!$C$5),0)</f>
         <v/>
       </c>
       <c r="O15" s="21" t="n"/>
@@ -2039,7 +2039,7 @@
         <v>57.88</v>
       </c>
       <c r="N16" s="9">
-        <f>IF(E16="UberXL",M16*(1+Resumen!$C$5),0)</f>
+        <f>IF(LEFT(E16,4)="Uber",M16*(1+Resumen!$C$5),0)</f>
         <v/>
       </c>
       <c r="O16" s="21" t="n"/>
@@ -2108,7 +2108,7 @@
         <v>57.88</v>
       </c>
       <c r="N17" s="9">
-        <f>IF(E17="UberXL",M17*(1+Resumen!$C$5),0)</f>
+        <f>IF(LEFT(E17,4)="Uber",M17*(1+Resumen!$C$5),0)</f>
         <v/>
       </c>
       <c r="O17" s="21" t="n"/>
@@ -2175,7 +2175,7 @@
         <v>47.51</v>
       </c>
       <c r="N18" s="9">
-        <f>IF(E18="UberXL",M18*(1+Resumen!$C$5),0)</f>
+        <f>IF(LEFT(E18,4)="Uber",M18*(1+Resumen!$C$5),0)</f>
         <v/>
       </c>
       <c r="O18" s="21" t="n"/>
@@ -2242,7 +2242,7 @@
         <v>0</v>
       </c>
       <c r="N19" s="9">
-        <f>IF(E19="UberXL",M19*(1+Resumen!$C$5),0)</f>
+        <f>IF(LEFT(E19,4)="Uber",M19*(1+Resumen!$C$5),0)</f>
         <v/>
       </c>
       <c r="O19" s="21" t="n"/>
@@ -2307,7 +2307,7 @@
         <v>51.87</v>
       </c>
       <c r="N20" s="9">
-        <f>IF(E20="UberXL",M20*(1+Resumen!$C$5),0)</f>
+        <f>IF(LEFT(E20,4)="Uber",M20*(1+Resumen!$C$5),0)</f>
         <v/>
       </c>
       <c r="O20" s="21" t="n"/>
@@ -2372,7 +2372,7 @@
         <v>50.1</v>
       </c>
       <c r="N21" s="9">
-        <f>IF(E21="UberXL",M21*(1+Resumen!$C$5),0)</f>
+        <f>IF(LEFT(E21,4)="Uber",M21*(1+Resumen!$C$5),0)</f>
         <v/>
       </c>
       <c r="O21" s="21" t="n"/>
@@ -2439,7 +2439,7 @@
         <v>47.51</v>
       </c>
       <c r="N22" s="9">
-        <f>IF(E22="UberXL",M22*(1+Resumen!$C$5),0)</f>
+        <f>IF(LEFT(E22,4)="Uber",M22*(1+Resumen!$C$5),0)</f>
         <v/>
       </c>
       <c r="O22" s="21" t="n"/>
@@ -2508,7 +2508,7 @@
         <v>123.28</v>
       </c>
       <c r="N23" s="9">
-        <f>IF(E23="UberXL",M23*(1+Resumen!$C$5),0)</f>
+        <f>IF(LEFT(E23,4)="Uber",M23*(1+Resumen!$C$5),0)</f>
         <v/>
       </c>
       <c r="O23" s="21" t="n"/>
@@ -2571,7 +2571,7 @@
         <v>0</v>
       </c>
       <c r="N24" s="9">
-        <f>IF(E24="UberXL",M24*(1+Resumen!$C$5),0)</f>
+        <f>IF(LEFT(E24,4)="Uber",M24*(1+Resumen!$C$5),0)</f>
         <v/>
       </c>
       <c r="O24" s="21" t="n"/>
@@ -2634,7 +2634,7 @@
         <v>129.03</v>
       </c>
       <c r="N25" s="9">
-        <f>IF(E25="UberXL",M25*(1+Resumen!$C$5),0)</f>
+        <f>IF(LEFT(E25,4)="Uber",M25*(1+Resumen!$C$5),0)</f>
         <v/>
       </c>
       <c r="O25" s="21" t="n"/>
@@ -2669,7 +2669,7 @@
       </c>
       <c r="E26" s="8" t="inlineStr">
         <is>
-          <t>UberXL</t>
+          <t>UberXXL</t>
         </is>
       </c>
       <c r="F26" s="18" t="n">
@@ -2696,10 +2696,10 @@
         <v>40</v>
       </c>
       <c r="M26" s="9" t="n">
-        <v>78.95999999999999</v>
+        <v>90.81</v>
       </c>
       <c r="N26" s="9">
-        <f>IF(E26="UberXL",M26*(1+Resumen!$C$5),0)</f>
+        <f>IF(LEFT(E26,4)="Uber",M26*(1+Resumen!$C$5),0)</f>
         <v/>
       </c>
       <c r="O26" s="21" t="n"/>

</xml_diff>